<commit_message>
Update commercial invoice template
</commit_message>
<xml_diff>
--- a/public/templates/commercial-invoice-template.xlsx
+++ b/public/templates/commercial-invoice-template.xlsx
@@ -3,13 +3,13 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="23040" windowHeight="9060" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="22188" windowHeight="9180" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="PI" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'PI'!$A$1:$I$24</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'PI'!$A$1:$I$31</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -21,7 +21,7 @@
     <numFmt numFmtId="164" formatCode="&quot;US$&quot;#,##0.00;\-&quot;US$&quot;#,##0.00"/>
     <numFmt numFmtId="165" formatCode="&quot;US$&quot;#,##0.00_);[Red]\(&quot;US$&quot;#,##0.00\)"/>
   </numFmts>
-  <fonts count="43">
+  <fonts count="45">
     <font>
       <name val="宋体"/>
       <charset val="134"/>
@@ -32,6 +32,12 @@
       <charset val="134"/>
       <b val="1"/>
       <sz val="16"/>
+    </font>
+    <font>
+      <name val="新細明體"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="新細明體"/>
@@ -68,7 +74,13 @@
       <name val="Calibri"/>
       <charset val="0"/>
       <color rgb="FF000000"/>
-      <sz val="11"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <color indexed="8"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -114,12 +126,12 @@
     <font>
       <name val="Calibri"/>
       <charset val="0"/>
-      <b val="1"/>
       <sz val="9"/>
     </font>
     <font>
       <name val="Calibri"/>
       <charset val="0"/>
+      <b val="1"/>
       <sz val="9"/>
     </font>
     <font>
@@ -132,6 +144,13 @@
       <name val="Calibri"/>
       <charset val="0"/>
       <color indexed="10"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <b val="1"/>
+      <color indexed="12"/>
       <sz val="9"/>
     </font>
     <font>
@@ -284,19 +303,19 @@
       <color indexed="8"/>
       <sz val="11"/>
     </font>
-    <font>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <color rgb="FFFF0000"/>
-      <sz val="9"/>
-    </font>
   </fonts>
-  <fills count="24">
+  <fills count="25">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -464,29 +483,12 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
+      <left/>
       <right/>
       <top style="thin">
         <color auto="1"/>
       </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
+      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -598,7 +600,9 @@
     </border>
     <border>
       <left/>
-      <right/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
       <top style="thin">
         <color auto="1"/>
       </top>
@@ -613,7 +617,20 @@
       <top style="thin">
         <color auto="1"/>
       </top>
-      <bottom/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -634,362 +651,369 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" applyAlignment="1" applyProtection="1">
       <alignment vertical="top"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" applyAlignment="1" applyProtection="1">
       <alignment vertical="top"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="6" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="7" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="8" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="3" borderId="9" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="4" borderId="10" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="4" borderId="9" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="5" borderId="11" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="12" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="13" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="6" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="38" fillId="7" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="8" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="40" fillId="9" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="10" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="11" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="40" fillId="12" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="40" fillId="13" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="7" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="14" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="40" fillId="14" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="40" fillId="15" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="6" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="16" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="40" fillId="16" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="40" fillId="17" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="18" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="18" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="40" fillId="17" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="40" fillId="19" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="20" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="11" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="40" fillId="19" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="40" fillId="21" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="3" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="22" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="40" fillId="23" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="5" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="6" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="7" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="4" borderId="8" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="5" borderId="9" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="5" borderId="8" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="6" borderId="10" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="11" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="12" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="7" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="8" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="9" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="10" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="11" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="12" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="13" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="14" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="8" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="15" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="15" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="16" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="7" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="17" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="17" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="18" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="19" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="19" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="18" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="20" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="21" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="12" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="20" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="22" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="4" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="23" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="24" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="89">
+  <cellXfs count="96">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="centerContinuous"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="centerContinuous"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="centerContinuous"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="centerContinuous"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="16" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="6">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="6">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="17" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="21" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="23" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="23" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="19" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="17" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="21" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="19" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="23" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="165" fontId="23" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -1308,495 +1332,426 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M30"/>
+  <dimension ref="A1:M35"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="15.6"/>
   <cols>
-    <col width="1.5" customWidth="1" min="1" max="1"/>
-    <col width="5.375" customWidth="1" min="2" max="2"/>
-    <col width="6.75" customWidth="1" min="3" max="3"/>
-    <col width="38.125" customWidth="1" min="4" max="4"/>
-    <col width="5.375" customWidth="1" min="5" max="5"/>
-    <col width="5.125" customWidth="1" min="6" max="6"/>
-    <col width="10.5" customWidth="1" min="7" max="7"/>
-    <col width="4.875" customWidth="1" min="8" max="8"/>
-    <col width="16.375" customWidth="1" min="9" max="9"/>
-    <col width="10.5" customWidth="1" min="11" max="11"/>
-    <col width="10.5" customWidth="1" min="13" max="13"/>
+    <col width="1.5" customWidth="1" style="8" min="1" max="1"/>
+    <col width="5.375" customWidth="1" style="8" min="2" max="2"/>
+    <col width="6.75" customWidth="1" style="8" min="3" max="3"/>
+    <col width="38.125" customWidth="1" style="8" min="4" max="4"/>
+    <col width="5.375" customWidth="1" style="8" min="5" max="5"/>
+    <col width="5.125" customWidth="1" style="8" min="6" max="6"/>
+    <col width="10.5" customWidth="1" style="8" min="7" max="7"/>
+    <col width="4.875" customWidth="1" style="8" min="8" max="8"/>
+    <col width="16.375" customWidth="1" style="8" min="9" max="9"/>
+    <col width="10.5" customWidth="1" style="8" min="11" max="11"/>
+    <col width="10.5" customWidth="1" style="8" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="26.25" customFormat="1" customHeight="1" s="1">
-      <c r="A1" s="7" t="inlineStr">
-        <is>
-          <t>GuangDong Jindaquan Technology Co.,Ltd</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="34" customFormat="1" customHeight="1" s="1">
-      <c r="A2" s="77" t="inlineStr">
-        <is>
-          <t>Room 1605, ShiHong Building, No. 2095 Bixin Road, Nanlian Community, Longgang Subdistrict, Longgang District, Shenzhen, Guangdong, China</t>
-        </is>
-      </c>
+      <c r="A1" s="10" t="n"/>
+    </row>
+    <row r="2" ht="18" customFormat="1" customHeight="1" s="2">
+      <c r="A2" s="11" t="n"/>
     </row>
     <row r="3" ht="18" customFormat="1" customHeight="1" s="1">
-      <c r="A3" s="9" t="n"/>
-      <c r="B3" s="9" t="n"/>
-      <c r="C3" s="9" t="n"/>
-      <c r="D3" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tel: +86-0755-28996208 </t>
-        </is>
-      </c>
-      <c r="E3" s="9" t="inlineStr">
-        <is>
-          <t>Fax: +86-0755-28994568</t>
-        </is>
-      </c>
-      <c r="H3" s="9" t="inlineStr">
+      <c r="A3" s="13" t="n"/>
+      <c r="B3" s="13" t="n"/>
+      <c r="C3" s="13" t="n"/>
+      <c r="D3" s="13" t="n"/>
+      <c r="E3" s="13" t="n"/>
+      <c r="H3" s="13" t="inlineStr">
         <is>
           <t> </t>
         </is>
       </c>
-      <c r="I3" s="9" t="n"/>
-    </row>
-    <row r="4" ht="21" customFormat="1" customHeight="1" s="2">
-      <c r="A4" s="10" t="n"/>
-      <c r="B4" s="11" t="n"/>
-      <c r="C4" s="12" t="n"/>
-      <c r="D4" s="12" t="inlineStr">
+      <c r="I3" s="13" t="n"/>
+    </row>
+    <row r="4" ht="21" customFormat="1" customHeight="1" s="3">
+      <c r="A4" s="14" t="n"/>
+      <c r="B4" s="15" t="inlineStr">
         <is>
           <t>COMMERCIAL INVOICE</t>
         </is>
       </c>
-      <c r="E4" s="13" t="n"/>
-      <c r="F4" s="13" t="n"/>
-      <c r="G4" s="13" t="n"/>
-      <c r="H4" s="12" t="n"/>
-      <c r="I4" s="12" t="n"/>
-    </row>
-    <row r="5" ht="24" customHeight="1">
-      <c r="A5" s="71" t="n"/>
-      <c r="B5" s="15" t="inlineStr">
+      <c r="C4" s="16" t="n"/>
+      <c r="D4" s="16" t="n"/>
+      <c r="E4" s="17" t="n"/>
+      <c r="F4" s="17" t="n"/>
+      <c r="G4" s="17" t="n"/>
+      <c r="H4" s="16" t="n"/>
+      <c r="I4" s="16" t="n"/>
+    </row>
+    <row r="5" ht="24" customHeight="1" s="8">
+      <c r="A5" s="69" t="n"/>
+      <c r="B5" s="19" t="inlineStr">
         <is>
           <t>Company:</t>
         </is>
       </c>
-      <c r="D5" s="16" t="inlineStr">
-        <is>
-          <t>Chawin Wanprasert ( Personal Buyer)</t>
-        </is>
-      </c>
-      <c r="E5" s="17" t="n"/>
-      <c r="F5" s="71" t="n"/>
-      <c r="G5" s="18" t="inlineStr">
-        <is>
-          <t>CI NO. :</t>
-        </is>
-      </c>
-      <c r="H5" s="67" t="inlineStr">
-        <is>
-          <t>ALL260609A01-THW01</t>
-        </is>
-      </c>
-      <c r="I5" s="67" t="n"/>
-    </row>
-    <row r="6" ht="26.25" customHeight="1">
-      <c r="A6" s="71" t="n"/>
-      <c r="B6" s="15" t="inlineStr">
+      <c r="D5" s="20" t="n"/>
+      <c r="E5" s="21" t="n"/>
+      <c r="F5" s="69" t="n"/>
+      <c r="G5" s="22" t="n"/>
+      <c r="H5" s="65" t="n"/>
+      <c r="I5" s="65" t="n"/>
+    </row>
+    <row r="6" ht="26.25" customHeight="1" s="8">
+      <c r="A6" s="69" t="n"/>
+      <c r="B6" s="19" t="inlineStr">
         <is>
           <t>ATTN:</t>
         </is>
       </c>
-      <c r="D6" s="16" t="inlineStr">
-        <is>
-          <t>Chawin Wanprasert</t>
-        </is>
-      </c>
-      <c r="E6" s="20" t="n"/>
-      <c r="F6" s="71" t="n"/>
-      <c r="G6" s="18" t="inlineStr">
+      <c r="D6" s="20" t="n"/>
+      <c r="E6" s="24" t="n"/>
+      <c r="F6" s="69" t="n"/>
+      <c r="G6" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">Date: </t>
         </is>
       </c>
-      <c r="H6" s="21" t="inlineStr">
-        <is>
-          <t>21/05/2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="33" customHeight="1">
-      <c r="A7" s="71" t="n"/>
-      <c r="B7" s="15" t="inlineStr">
+      <c r="H6" s="25" t="n"/>
+    </row>
+    <row r="7" ht="33" customFormat="1" customHeight="1" s="4">
+      <c r="A7" s="61" t="n"/>
+      <c r="B7" s="19" t="inlineStr">
         <is>
           <t>Add.</t>
         </is>
       </c>
-      <c r="D7" s="22" t="inlineStr">
-        <is>
-          <t>480/63 Venezia Residence Phetburi 18 Ratchathewi Bangkok 10400, Thailand</t>
-        </is>
-      </c>
-      <c r="E7" s="20" t="n"/>
-      <c r="F7" s="71" t="n"/>
-      <c r="G7" s="15" t="inlineStr">
+      <c r="D7" s="27" t="n"/>
+      <c r="E7" s="28" t="n"/>
+      <c r="F7" s="61" t="n"/>
+      <c r="G7" s="19" t="inlineStr">
         <is>
           <t>By:</t>
         </is>
       </c>
-      <c r="H7" s="23" t="inlineStr">
-        <is>
-          <t>ALEX GONG</t>
-        </is>
-      </c>
-      <c r="I7" s="23" t="n"/>
-      <c r="J7" t="inlineStr">
+      <c r="H7" s="19" t="n"/>
+      <c r="I7" s="19" t="n"/>
+      <c r="J7" s="4" t="inlineStr">
         <is>
           <t> </t>
         </is>
       </c>
     </row>
-    <row r="8" ht="22.5" customHeight="1">
-      <c r="A8" s="71" t="n"/>
-      <c r="B8" s="24" t="inlineStr">
+    <row r="8" ht="22.5" customHeight="1" s="8">
+      <c r="A8" s="69" t="n"/>
+      <c r="B8" s="29" t="inlineStr">
         <is>
           <t>Tel:</t>
         </is>
       </c>
-      <c r="C8" s="78" t="n"/>
-      <c r="D8" s="25" t="inlineStr">
-        <is>
-          <t>+66 0840014483</t>
-        </is>
-      </c>
-      <c r="E8" s="20" t="n"/>
-      <c r="F8" s="23" t="inlineStr">
+      <c r="C8" s="84" t="n"/>
+      <c r="D8" s="30" t="n"/>
+      <c r="E8" s="24" t="n"/>
+      <c r="F8" s="31" t="inlineStr">
         <is>
           <t xml:space="preserve">From:                         </t>
         </is>
       </c>
-      <c r="G8" s="64" t="inlineStr">
-        <is>
-          <t>China</t>
-        </is>
-      </c>
-      <c r="H8" s="27" t="inlineStr">
+      <c r="G8" s="62" t="n"/>
+      <c r="H8" s="33" t="inlineStr">
         <is>
           <t>To</t>
         </is>
       </c>
-      <c r="I8" s="28" t="inlineStr">
-        <is>
-          <t>Thailand</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="29" customFormat="1" customHeight="1" s="3">
-      <c r="A9" s="29" t="n"/>
-      <c r="B9" s="30" t="inlineStr">
+      <c r="I8" s="34" t="n"/>
+    </row>
+    <row r="9" ht="29" customFormat="1" customHeight="1" s="5">
+      <c r="A9" s="35" t="n"/>
+      <c r="B9" s="36" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="C9" s="30" t="inlineStr">
+      <c r="C9" s="36" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="D9" s="79" t="n"/>
-      <c r="E9" s="30" t="inlineStr">
+      <c r="D9" s="85" t="n"/>
+      <c r="E9" s="36" t="inlineStr">
         <is>
           <t>QTY(KG)</t>
         </is>
       </c>
-      <c r="F9" s="79" t="n"/>
-      <c r="G9" s="31" t="inlineStr">
+      <c r="F9" s="85" t="n"/>
+      <c r="G9" s="37" t="inlineStr">
         <is>
           <t>Unit Price
 (EXW)</t>
         </is>
       </c>
-      <c r="H9" s="79" t="n"/>
-      <c r="I9" s="30" t="inlineStr">
+      <c r="H9" s="85" t="n"/>
+      <c r="I9" s="36" t="inlineStr">
         <is>
           <t>Subtotal</t>
         </is>
       </c>
-      <c r="K9" s="5" t="n"/>
-      <c r="M9" s="5" t="n"/>
-    </row>
-    <row r="10" ht="18" customFormat="1" customHeight="1" s="5">
-      <c r="A10" s="51" t="n"/>
-      <c r="B10" s="36" t="n">
-        <v>1</v>
-      </c>
-      <c r="C10" s="34" t="inlineStr">
-        <is>
-          <t>Plastic granules (HS CODE:2917140000)</t>
-        </is>
-      </c>
-      <c r="D10" s="79" t="n"/>
-      <c r="E10" s="36" t="inlineStr">
-        <is>
-          <t>5KG</t>
-        </is>
-      </c>
-      <c r="F10" s="79" t="n"/>
-      <c r="G10" s="80" t="n">
-        <v>3.9</v>
-      </c>
-      <c r="H10" s="79" t="n"/>
-      <c r="I10" s="81" t="n">
-        <v>19.5</v>
-      </c>
-      <c r="K10" s="5" t="n"/>
-      <c r="M10" s="5" t="n"/>
-    </row>
-    <row r="11" ht="19" customFormat="1" customHeight="1" s="5">
-      <c r="A11" s="51" t="n"/>
-      <c r="B11" s="36" t="n">
-        <v>2</v>
-      </c>
-      <c r="C11" s="34" t="inlineStr">
-        <is>
-          <t>Plastic granules (HS CODE:3902100090)</t>
-        </is>
-      </c>
-      <c r="D11" s="79" t="n"/>
-      <c r="E11" s="36" t="inlineStr">
-        <is>
-          <t>5kg</t>
-        </is>
-      </c>
-      <c r="F11" s="79" t="n"/>
-      <c r="G11" s="80" t="inlineStr">
-        <is>
-          <t>3.5$</t>
-        </is>
-      </c>
-      <c r="H11" s="79" t="n"/>
-      <c r="I11" s="81" t="n">
-        <v>17.5</v>
-      </c>
-      <c r="K11" s="5" t="n"/>
-      <c r="M11" s="5" t="n"/>
-    </row>
-    <row r="12" ht="19" customFormat="1" customHeight="1" s="5">
-      <c r="A12" s="51" t="n"/>
-      <c r="B12" s="36" t="n">
-        <v>3</v>
-      </c>
-      <c r="C12" s="34" t="inlineStr">
-        <is>
-          <t>Shipping Fee</t>
-        </is>
-      </c>
-      <c r="D12" s="79" t="n"/>
-      <c r="E12" s="36" t="inlineStr">
-        <is>
-          <t>***</t>
-        </is>
-      </c>
-      <c r="F12" s="79" t="n"/>
-      <c r="G12" s="80" t="inlineStr">
-        <is>
-          <t>***</t>
-        </is>
-      </c>
-      <c r="H12" s="79" t="n"/>
-      <c r="I12" s="81" t="n">
-        <v>106</v>
-      </c>
-      <c r="K12" s="5" t="n"/>
-      <c r="M12" s="5" t="n"/>
-    </row>
-    <row r="13" ht="19" customFormat="1" customHeight="1" s="5">
-      <c r="A13" s="51" t="n"/>
-      <c r="B13" s="36" t="n">
-        <v>4</v>
-      </c>
-      <c r="C13" s="34" t="inlineStr">
-        <is>
-          <t>Bank transfer fee</t>
-        </is>
-      </c>
-      <c r="D13" s="79" t="n"/>
-      <c r="E13" s="36" t="inlineStr">
-        <is>
-          <t>***</t>
-        </is>
-      </c>
-      <c r="F13" s="79" t="n"/>
-      <c r="G13" s="80" t="inlineStr">
-        <is>
-          <t>***</t>
-        </is>
-      </c>
-      <c r="H13" s="79" t="n"/>
-      <c r="I13" s="81" t="n">
-        <v>25</v>
-      </c>
-      <c r="K13" s="5" t="n"/>
-      <c r="M13" s="5" t="n"/>
-    </row>
-    <row r="14" ht="19" customFormat="1" customHeight="1" s="5">
-      <c r="A14" s="51" t="n"/>
-      <c r="B14" s="36" t="n"/>
-      <c r="C14" s="34" t="n"/>
-      <c r="D14" s="79" t="n"/>
-      <c r="E14" s="36" t="n"/>
-      <c r="F14" s="79" t="n"/>
-      <c r="G14" s="80" t="n"/>
-      <c r="H14" s="79" t="n"/>
-      <c r="I14" s="81" t="n">
-        <v>168</v>
-      </c>
-      <c r="K14" s="5" t="n"/>
-      <c r="M14" s="5" t="n"/>
-    </row>
-    <row r="15" ht="24" customFormat="1" customHeight="1" s="5">
-      <c r="A15" s="51" t="n"/>
-      <c r="B15" s="52" t="n"/>
-      <c r="J15" s="82" t="n"/>
-      <c r="K15" s="82" t="n"/>
-      <c r="L15" s="82" t="n"/>
-    </row>
-    <row r="16" ht="16" customFormat="1" customHeight="1" s="5">
-      <c r="A16" s="51" t="n"/>
-      <c r="B16" s="54" t="n"/>
-      <c r="D16" s="55" t="n"/>
-      <c r="K16" s="82" t="n"/>
-    </row>
-    <row r="17" ht="21" customFormat="1" customHeight="1" s="5">
-      <c r="A17" s="51" t="n"/>
-      <c r="B17" s="54" t="n"/>
-      <c r="D17" s="56" t="n"/>
-      <c r="E17" s="57" t="n"/>
-      <c r="F17" s="83" t="n"/>
-      <c r="G17" s="59" t="n"/>
-      <c r="H17" s="56" t="n"/>
-      <c r="I17" s="84" t="n"/>
-    </row>
-    <row r="18" ht="2" customHeight="1">
-      <c r="A18" s="71" t="n"/>
-      <c r="B18" s="61" t="n"/>
-      <c r="C18" s="61" t="n"/>
-      <c r="D18" s="64" t="n"/>
-      <c r="E18" s="23" t="n"/>
-      <c r="F18" s="85" t="n"/>
-      <c r="G18" s="63" t="n"/>
-      <c r="H18" s="64" t="n"/>
-      <c r="I18" s="86" t="n"/>
+      <c r="K9" s="7" t="n"/>
+      <c r="M9" s="7" t="n"/>
+    </row>
+    <row r="10" ht="18" customFormat="1" customHeight="1" s="7">
+      <c r="A10" s="45" t="n"/>
+      <c r="B10" s="42" t="n"/>
+      <c r="C10" s="40" t="n"/>
+      <c r="D10" s="85" t="n"/>
+      <c r="E10" s="42" t="n"/>
+      <c r="F10" s="85" t="n"/>
+      <c r="G10" s="86" t="n"/>
+      <c r="H10" s="85" t="n"/>
+      <c r="I10" s="87" t="n"/>
+      <c r="K10" s="7" t="n"/>
+      <c r="M10" s="7" t="n"/>
+    </row>
+    <row r="11" ht="16" customFormat="1" customHeight="1" s="7">
+      <c r="A11" s="45" t="n"/>
+      <c r="B11" s="42" t="n"/>
+      <c r="C11" s="40" t="n"/>
+      <c r="D11" s="85" t="n"/>
+      <c r="E11" s="42" t="n"/>
+      <c r="F11" s="85" t="n"/>
+      <c r="G11" s="86" t="n"/>
+      <c r="H11" s="85" t="n"/>
+      <c r="I11" s="87" t="n"/>
+      <c r="K11" s="7" t="n"/>
+      <c r="M11" s="7" t="n"/>
+    </row>
+    <row r="12" ht="22" customFormat="1" customHeight="1" s="7">
+      <c r="A12" s="45" t="n"/>
+      <c r="B12" s="42" t="n"/>
+      <c r="C12" s="40" t="n"/>
+      <c r="D12" s="85" t="n"/>
+      <c r="E12" s="42" t="n"/>
+      <c r="F12" s="85" t="n"/>
+      <c r="G12" s="86" t="n"/>
+      <c r="H12" s="85" t="n"/>
+      <c r="I12" s="87" t="n"/>
+      <c r="K12" s="7" t="n"/>
+      <c r="M12" s="7" t="n"/>
+    </row>
+    <row r="13" ht="18" customFormat="1" customHeight="1" s="7">
+      <c r="A13" s="45" t="n"/>
+      <c r="B13" s="42" t="n"/>
+      <c r="C13" s="40" t="n"/>
+      <c r="D13" s="85" t="n"/>
+      <c r="E13" s="42" t="n"/>
+      <c r="F13" s="85" t="n"/>
+      <c r="G13" s="86" t="n"/>
+      <c r="H13" s="85" t="n"/>
+      <c r="I13" s="87" t="n"/>
+      <c r="K13" s="7" t="n"/>
+      <c r="M13" s="7" t="n"/>
+    </row>
+    <row r="14" ht="18" customFormat="1" customHeight="1" s="7">
+      <c r="A14" s="45" t="n"/>
+      <c r="B14" s="46" t="n"/>
+      <c r="C14" s="88" t="n"/>
+      <c r="D14" s="85" t="n"/>
+      <c r="E14" s="48" t="n"/>
+      <c r="F14" s="85" t="n"/>
+      <c r="G14" s="48" t="n"/>
+      <c r="H14" s="85" t="n"/>
+      <c r="I14" s="89" t="n"/>
+      <c r="K14" s="90" t="n"/>
+    </row>
+    <row r="15" ht="24" customFormat="1" customHeight="1" s="7">
+      <c r="A15" s="45" t="n"/>
+      <c r="B15" s="51" t="n"/>
+      <c r="J15" s="90" t="n"/>
+      <c r="K15" s="90" t="n"/>
+      <c r="L15" s="90" t="n"/>
+    </row>
+    <row r="16" ht="16" customFormat="1" customHeight="1" s="7">
+      <c r="A16" s="45" t="n"/>
+      <c r="B16" s="52" t="n"/>
+      <c r="D16" s="74" t="n"/>
+      <c r="K16" s="90" t="n"/>
+    </row>
+    <row r="17" ht="21" customFormat="1" customHeight="1" s="7">
+      <c r="A17" s="45" t="n"/>
+      <c r="B17" s="52" t="n"/>
+      <c r="D17" s="75" t="n"/>
+      <c r="E17" s="55" t="n"/>
+      <c r="F17" s="91" t="n"/>
+      <c r="G17" s="57" t="n"/>
+      <c r="H17" s="75" t="n"/>
+      <c r="I17" s="92" t="n"/>
+    </row>
+    <row r="18" ht="2" customHeight="1" s="8">
+      <c r="A18" s="69" t="n"/>
+      <c r="B18" s="59" t="n"/>
+      <c r="C18" s="59" t="n"/>
+      <c r="D18" s="62" t="n"/>
+      <c r="E18" s="31" t="n"/>
+      <c r="F18" s="93" t="n"/>
+      <c r="G18" s="61" t="n"/>
+      <c r="H18" s="62" t="n"/>
+      <c r="I18" s="94" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="71" t="n"/>
-      <c r="B19" s="67" t="n"/>
-      <c r="C19" s="67" t="n"/>
-      <c r="D19" s="68" t="n"/>
-      <c r="E19" s="87" t="n"/>
-      <c r="F19" s="70" t="n"/>
-      <c r="G19" s="71" t="n"/>
-      <c r="H19" s="71" t="n"/>
-      <c r="I19" s="71" t="n"/>
-    </row>
-    <row r="20" ht="23.1" customHeight="1">
-      <c r="A20" s="71" t="n"/>
-      <c r="B20" s="71" t="n"/>
-      <c r="C20" s="64" t="inlineStr">
-        <is>
-          <t>The seller</t>
-        </is>
-      </c>
+      <c r="A19" s="69" t="n"/>
+      <c r="B19" s="65" t="n"/>
+      <c r="C19" s="65" t="n"/>
+      <c r="D19" s="66" t="n"/>
+      <c r="E19" s="95" t="n"/>
+      <c r="F19" s="68" t="n"/>
+      <c r="G19" s="69" t="n"/>
+      <c r="H19" s="69" t="n"/>
+      <c r="I19" s="69" t="n"/>
+    </row>
+    <row r="20" ht="18" customHeight="1" s="8">
+      <c r="A20" s="69" t="n"/>
+      <c r="B20" s="70" t="n"/>
+      <c r="C20" s="71" t="n"/>
       <c r="D20" s="71" t="n"/>
       <c r="E20" s="71" t="n"/>
-      <c r="F20" s="71" t="n"/>
-      <c r="G20" s="64" t="inlineStr">
-        <is>
-          <t>The buyer</t>
-        </is>
-      </c>
+      <c r="F20" s="70" t="n"/>
+      <c r="G20" s="71" t="n"/>
       <c r="H20" s="71" t="n"/>
-      <c r="I20" s="71" t="n"/>
-    </row>
-    <row r="21" ht="54" customHeight="1">
-      <c r="A21" s="71" t="n"/>
-      <c r="B21" s="71" t="n"/>
-      <c r="C21" s="72" t="inlineStr">
-        <is>
-          <t>Guangdong Jindaquan Technology Co.,Ltd</t>
-        </is>
-      </c>
-      <c r="D21" s="71" t="n"/>
-      <c r="E21" s="71" t="n"/>
-      <c r="F21" s="71" t="n"/>
-      <c r="G21" s="72">
-        <f>D5</f>
-        <v/>
-      </c>
-      <c r="H21" s="71" t="n"/>
-      <c r="I21" s="71" t="n"/>
-    </row>
-    <row r="23">
-      <c r="B23" s="88" t="n"/>
-    </row>
-    <row r="24" ht="24" customHeight="1">
-      <c r="A24" s="71" t="n"/>
-      <c r="B24" s="16" t="n"/>
-      <c r="C24" s="71" t="n"/>
-      <c r="D24" t="inlineStr">
+      <c r="I20" s="72" t="n"/>
+      <c r="J20" s="73" t="n"/>
+      <c r="K20" s="69" t="n"/>
+    </row>
+    <row r="21" ht="20" customHeight="1" s="8">
+      <c r="A21" s="69" t="n"/>
+      <c r="B21" s="74" t="n"/>
+      <c r="J21" s="73" t="n"/>
+      <c r="K21" s="69" t="n"/>
+    </row>
+    <row r="22" ht="16" customHeight="1" s="8">
+      <c r="A22" s="69" t="n"/>
+      <c r="B22" s="75" t="n"/>
+      <c r="C22" s="45" t="n"/>
+      <c r="D22" s="45" t="n"/>
+      <c r="E22" s="45" t="n"/>
+      <c r="F22" s="75" t="n"/>
+      <c r="G22" s="45" t="n"/>
+      <c r="H22" s="45" t="n"/>
+      <c r="I22" s="7" t="n"/>
+      <c r="J22" s="73" t="n"/>
+      <c r="K22" s="69" t="n"/>
+    </row>
+    <row r="23" ht="15" customHeight="1" s="8">
+      <c r="A23" s="69" t="n"/>
+      <c r="B23" s="75" t="n"/>
+      <c r="C23" s="45" t="n"/>
+      <c r="D23" s="45" t="n"/>
+      <c r="E23" s="45" t="n"/>
+      <c r="F23" s="75" t="n"/>
+      <c r="G23" s="45" t="n"/>
+      <c r="H23" s="45" t="n"/>
+      <c r="I23" s="7" t="n"/>
+      <c r="J23" s="73" t="n"/>
+      <c r="K23" s="69" t="n"/>
+    </row>
+    <row r="24" ht="15" customHeight="1" s="8">
+      <c r="A24" s="69" t="n"/>
+      <c r="B24" s="75" t="n"/>
+      <c r="C24" s="45" t="n"/>
+      <c r="D24" s="45" t="n"/>
+      <c r="E24" s="45" t="n"/>
+      <c r="F24" s="75" t="n"/>
+      <c r="G24" s="45" t="n"/>
+      <c r="H24" s="45" t="n"/>
+      <c r="I24" s="7" t="n"/>
+      <c r="J24" s="73" t="n"/>
+      <c r="K24" s="69" t="n"/>
+    </row>
+    <row r="25" ht="23" customHeight="1" s="8">
+      <c r="A25" s="69" t="n"/>
+      <c r="B25" s="76" t="n"/>
+      <c r="C25" s="77" t="n"/>
+      <c r="D25" s="77" t="n"/>
+      <c r="E25" s="77" t="n"/>
+      <c r="F25" s="76" t="n"/>
+      <c r="G25" s="77" t="n"/>
+      <c r="H25" s="77" t="n"/>
+      <c r="I25" s="78" t="n"/>
+      <c r="J25" s="73" t="n"/>
+      <c r="K25" s="69" t="n"/>
+    </row>
+    <row r="26"/>
+    <row r="27" ht="23.1" customHeight="1" s="8">
+      <c r="A27" s="69" t="n"/>
+      <c r="B27" s="69" t="n"/>
+      <c r="C27" s="62" t="n"/>
+      <c r="D27" s="69" t="n"/>
+      <c r="E27" s="69" t="n"/>
+      <c r="F27" s="69" t="n"/>
+      <c r="G27" s="62" t="n"/>
+      <c r="H27" s="69" t="n"/>
+      <c r="I27" s="69" t="n"/>
+    </row>
+    <row r="28" ht="54" customHeight="1" s="8">
+      <c r="A28" s="69" t="n"/>
+      <c r="B28" s="69" t="n"/>
+      <c r="C28" s="79" t="n"/>
+      <c r="D28" s="69" t="n"/>
+      <c r="E28" s="69" t="n"/>
+      <c r="F28" s="69" t="n"/>
+      <c r="G28" s="79" t="n"/>
+      <c r="H28" s="69" t="n"/>
+      <c r="I28" s="69" t="n"/>
+    </row>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31" ht="24" customHeight="1" s="8">
+      <c r="A31" s="69" t="n"/>
+      <c r="B31" s="69" t="n"/>
+      <c r="C31" s="69" t="n"/>
+      <c r="D31" t="inlineStr">
         <is>
           <t> </t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="E31" t="inlineStr">
         <is>
           <t> </t>
         </is>
       </c>
-      <c r="F24" s="71" t="n"/>
-      <c r="G24" s="71" t="n"/>
-      <c r="H24" s="71" t="n"/>
-      <c r="I24" s="71" t="n"/>
-    </row>
-    <row r="25" ht="42.95" customHeight="1">
-      <c r="A25" s="71" t="n"/>
-      <c r="B25" s="73" t="n"/>
-    </row>
-    <row r="26" ht="27.75" customFormat="1" customHeight="1" s="6">
-      <c r="A26" s="76" t="n"/>
-      <c r="H26" s="88" t="n"/>
-    </row>
-    <row r="27" ht="27.75" customFormat="1" customHeight="1" s="6">
-      <c r="A27" s="76" t="n"/>
-      <c r="H27" s="88" t="n"/>
-    </row>
-    <row r="28" ht="27.75" customFormat="1" customHeight="1" s="6">
-      <c r="A28" s="76" t="n"/>
-      <c r="H28" s="88" t="n"/>
-    </row>
-    <row r="29"/>
-    <row r="30"/>
+      <c r="F31" s="69" t="n"/>
+      <c r="G31" s="69" t="n"/>
+      <c r="H31" s="69" t="n"/>
+      <c r="I31" s="69" t="n"/>
+    </row>
+    <row r="32" ht="42.95" customHeight="1" s="8">
+      <c r="A32" s="69" t="n"/>
+      <c r="B32" s="80" t="n"/>
+    </row>
+    <row r="33" ht="27.75" customFormat="1" customHeight="1" s="9">
+      <c r="A33" s="83" t="n"/>
+    </row>
+    <row r="34" ht="27.75" customFormat="1" customHeight="1" s="9">
+      <c r="A34" s="83" t="n"/>
+    </row>
+    <row r="35" ht="27.75" customFormat="1" customHeight="1" s="9">
+      <c r="A35" s="83" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="34">
+  <mergeCells count="35">
     <mergeCell ref="E12:F12"/>
     <mergeCell ref="G12:H12"/>
+    <mergeCell ref="B14:D14"/>
     <mergeCell ref="B16:C16"/>
     <mergeCell ref="B7:C7"/>
-    <mergeCell ref="B25:I25"/>
     <mergeCell ref="G11:H11"/>
-    <mergeCell ref="C14:D14"/>
+    <mergeCell ref="A35:G35"/>
     <mergeCell ref="E14:F14"/>
     <mergeCell ref="D16:I16"/>
-    <mergeCell ref="A28:G28"/>
+    <mergeCell ref="B21:I21"/>
     <mergeCell ref="A2:I2"/>
     <mergeCell ref="H6:I6"/>
     <mergeCell ref="C10:D10"/>
     <mergeCell ref="E10:F10"/>
     <mergeCell ref="G10:H10"/>
+    <mergeCell ref="A34:G34"/>
     <mergeCell ref="E13:F13"/>
-    <mergeCell ref="B17:C17"/>
     <mergeCell ref="C9:D9"/>
     <mergeCell ref="G13:H13"/>
+    <mergeCell ref="B17:C17"/>
     <mergeCell ref="E9:F9"/>
     <mergeCell ref="B8:C8"/>
     <mergeCell ref="C12:D12"/>
@@ -1806,12 +1761,12 @@
     <mergeCell ref="E3:G3"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B15:I15"/>
-    <mergeCell ref="A27:G27"/>
     <mergeCell ref="B5:C5"/>
     <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A26:G26"/>
     <mergeCell ref="C13:D13"/>
     <mergeCell ref="G9:H9"/>
+    <mergeCell ref="A33:G33"/>
+    <mergeCell ref="B32:I32"/>
   </mergeCells>
   <pageMargins left="0.12" right="0.12" top="0.75" bottom="0.9399999999999999" header="0" footer="0.31"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="1200" verticalDpi="1200"/>

</xml_diff>